<commit_message>
Update pecan second-round watering workbook
</commit_message>
<xml_diff>
--- a/data/tree_and_watering_data/Pecan_Data_Second_Round_May-July.xlsx
+++ b/data/tree_and_watering_data/Pecan_Data_Second_Round_May-July.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e5e73ff6e8b2309b/Documents/SourceCode/Photo3-Plant-Salinity-Traits/data/tree_and_watering_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="11_D14B78FB1B9376EB9C7112035A75A356C5BBED09" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEC2A9B4-8775-4966-B2F3-F76BF3322C03}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="11_D14B78FB1B9376EB9C7112035A75A356C5BBED09" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBB9D480-E0F8-470B-846F-80E209ED0D80}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Watering Chart" sheetId="1" r:id="rId1"/>
@@ -439,8 +439,8 @@
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="#,##0.000"/>
-    <numFmt numFmtId="167" formatCode="#,##0.00000"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0000000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00000"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0000000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -708,10 +708,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -729,6 +729,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -48413,7 +48417,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E1000"/>
+  <dimension ref="A1:H1000"/>
   <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -48424,7 +48428,7 @@
     <col min="6" max="26" width="8.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="55.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" ht="55.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="11" t="s">
         <v>2</v>
       </c>
@@ -48439,7 +48443,7 @@
       </c>
       <c r="E1" s="26"/>
     </row>
-    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="29" t="s">
         <v>46</v>
       </c>
@@ -48453,8 +48457,12 @@
         <v>4318</v>
       </c>
       <c r="E2" s="27"/>
-    </row>
-    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="H2">
+        <f>(0.01/4)*1000</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="29" t="s">
         <v>49</v>
       </c>
@@ -48469,7 +48477,7 @@
       </c>
       <c r="E3" s="26"/>
     </row>
-    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="29" t="s">
         <v>50</v>
       </c>
@@ -48484,7 +48492,7 @@
       </c>
       <c r="E4" s="26"/>
     </row>
-    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="29" t="s">
         <v>51</v>
       </c>
@@ -48499,7 +48507,7 @@
       </c>
       <c r="E5" s="26"/>
     </row>
-    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="29" t="s">
         <v>52</v>
       </c>
@@ -48514,7 +48522,7 @@
       </c>
       <c r="E6" s="26"/>
     </row>
-    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="29" t="s">
         <v>53</v>
       </c>
@@ -48529,7 +48537,7 @@
       </c>
       <c r="E7" s="26"/>
     </row>
-    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="29" t="s">
         <v>54</v>
       </c>
@@ -48544,7 +48552,7 @@
       </c>
       <c r="E8" s="26"/>
     </row>
-    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="29" t="s">
         <v>55</v>
       </c>
@@ -48559,7 +48567,7 @@
       </c>
       <c r="E9" s="26"/>
     </row>
-    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="29" t="s">
         <v>56</v>
       </c>
@@ -48574,7 +48582,7 @@
       </c>
       <c r="E10" s="26"/>
     </row>
-    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="29" t="s">
         <v>57</v>
       </c>
@@ -48589,7 +48597,7 @@
       </c>
       <c r="E11" s="26"/>
     </row>
-    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="29" t="s">
         <v>58</v>
       </c>
@@ -48604,7 +48612,7 @@
       </c>
       <c r="E12" s="26"/>
     </row>
-    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="29" t="s">
         <v>59</v>
       </c>
@@ -48619,7 +48627,7 @@
       </c>
       <c r="E13" s="26"/>
     </row>
-    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="29" t="s">
         <v>60</v>
       </c>
@@ -48634,7 +48642,7 @@
       </c>
       <c r="E14" s="26"/>
     </row>
-    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="29" t="s">
         <v>61</v>
       </c>
@@ -48649,7 +48657,7 @@
       </c>
       <c r="E15" s="26"/>
     </row>
-    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="29" t="s">
         <v>62</v>
       </c>

</xml_diff>